<commit_message>
Updated website dashboard analysis.
</commit_message>
<xml_diff>
--- a/dashboard/Website-Performance-Dashboard.xlsx
+++ b/dashboard/Website-Performance-Dashboard.xlsx
@@ -1,29 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/916b396f8520dbf6/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="314" documentId="8_{D87F9695-6720-4733-8926-8BB5FA56CC3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4144D27E-9A32-4955-BFF1-EB1EEF1BB566}"/>
+  <xr:revisionPtr revIDLastSave="464" documentId="8_{D87F9695-6720-4733-8926-8BB5FA56CC3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{125E61E8-E159-4437-BC8F-4F5A5B3812F4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{59527EBC-376C-48C6-803F-5CE0B4691CF2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{59527EBC-376C-48C6-803F-5CE0B4691CF2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="4" state="hidden" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="4" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="5" state="hidden" r:id="rId2"/>
     <sheet name="Sheet4" sheetId="6" state="hidden" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="Slicer_Source">#N/A</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+      <x14:slicerCaches>
+        <x14:slicerCache r:id="rId7"/>
+      </x14:slicerCaches>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -180,7 +191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -200,6 +211,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -207,6 +219,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -243,13 +260,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="95000"/>
                   </a:schemeClr>
                 </a:solidFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                    <a:prstClr val="black">
+                      <a:alpha val="40000"/>
+                    </a:prstClr>
+                  </a:outerShdw>
+                </a:effectLst>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
@@ -262,14 +285,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.25148600174978125"/>
-          <c:y val="0.11472003499562555"/>
-        </c:manualLayout>
-      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -283,13 +298,19 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
                 </a:schemeClr>
               </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -303,17 +324,104 @@
     <c:pivotFmts>
       <c:pivotFmt>
         <c:idx val="0"/>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
         <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
+          <a:gradFill rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="accent1">
+                  <a:satMod val="103000"/>
+                  <a:lumMod val="102000"/>
+                  <a:tint val="94000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="50000">
+                <a:schemeClr val="accent1">
+                  <a:satMod val="110000"/>
+                  <a:lumMod val="100000"/>
+                  <a:shade val="100000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="99000"/>
+                  <a:satMod val="120000"/>
+                  <a:shade val="78000"/>
+                </a:schemeClr>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="5400000" scaled="0"/>
+          </a:gradFill>
           <a:ln>
             <a:noFill/>
           </a:ln>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="none"/>
+          <c:symbol val="diamond"/>
+          <c:size val="5"/>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -333,66 +441,8 @@
               <a:pPr>
                 <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="1"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
+                    <a:schemeClr val="lt1">
+                      <a:lumMod val="85000"/>
                     </a:schemeClr>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
@@ -447,13 +497,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
@@ -473,9 +552,8 @@
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
+                      <a:schemeClr val="lt1">
+                        <a:lumMod val="85000"/>
                       </a:schemeClr>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
@@ -499,14 +577,13 @@
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                    <a:ln w="9525">
                       <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
+                        <a:schemeClr val="lt1">
+                          <a:lumMod val="95000"/>
+                          <a:alpha val="54000"/>
                         </a:schemeClr>
                       </a:solidFill>
-                      <a:round/>
                     </a:ln>
                     <a:effectLst/>
                   </c:spPr>
@@ -558,7 +635,8 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="182"/>
+        <c:gapWidth val="115"/>
+        <c:overlap val="-20"/>
         <c:axId val="1456010016"/>
         <c:axId val="1456010496"/>
       </c:barChart>
@@ -570,16 +648,16 @@
         <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -593,9 +671,8 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -621,7 +698,7 @@
         <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -638,9 +715,8 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -663,37 +739,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -706,17 +751,28 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
     </a:ln>
     <a:effectLst/>
   </c:spPr>
@@ -741,7 +797,6 @@
         <c14:dropZoneFilter val="1"/>
         <c14:dropZoneCategories val="1"/>
         <c14:dropZoneData val="1"/>
-        <c14:dropZoneSeries val="1"/>
         <c14:dropZonesVisible val="1"/>
       </c14:pivotOptions>
     </c:ext>
@@ -779,13 +834,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="95000"/>
                   </a:schemeClr>
                 </a:solidFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                    <a:prstClr val="black">
+                      <a:alpha val="40000"/>
+                    </a:prstClr>
+                  </a:outerShdw>
+                </a:effectLst>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
@@ -793,13 +854,8 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-IN"/>
-              <a:t>Monthly</a:t>
+              <a:t>Monthly Sessions Trend</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="en-IN" baseline="0"/>
-              <a:t> Sessions Trend</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-IN"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -816,13 +872,19 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
                 </a:schemeClr>
               </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -836,20 +898,104 @@
     <c:pivotFmts>
       <c:pivotFmt>
         <c:idx val="0"/>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:dLblPos val="t"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
         <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln w="28575" cap="rnd">
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:round/>
+          <a:gradFill rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="accent6">
+                  <a:satMod val="103000"/>
+                  <a:lumMod val="102000"/>
+                  <a:tint val="94000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="50000">
+                <a:schemeClr val="accent6">
+                  <a:satMod val="110000"/>
+                  <a:lumMod val="100000"/>
+                  <a:shade val="100000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="99000"/>
+                  <a:satMod val="120000"/>
+                  <a:shade val="78000"/>
+                </a:schemeClr>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="5400000" scaled="0"/>
+          </a:gradFill>
+          <a:ln>
+            <a:noFill/>
           </a:ln>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="none"/>
+          <c:symbol val="circle"/>
+          <c:size val="6"/>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent6">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent6">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -869,9 +1015,8 @@
               <a:pPr>
                 <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
+                    <a:schemeClr val="lt1">
+                      <a:lumMod val="85000"/>
                     </a:schemeClr>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
@@ -882,64 +1027,6 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="t"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="1"/>
-        <c:spPr>
-          <a:ln w="28575" cap="rnd">
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="1"/>
           <c:showCatName val="0"/>
@@ -954,8 +1041,9 @@
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
@@ -972,17 +1060,44 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent6">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent6">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
+          <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:spPr>
               <a:noFill/>
@@ -1000,9 +1115,8 @@
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
+                      <a:schemeClr val="lt1">
+                        <a:lumMod val="85000"/>
                       </a:schemeClr>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
@@ -1013,7 +1127,6 @@
                 <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
-            <c:dLblPos val="t"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -1026,14 +1139,13 @@
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                    <a:ln w="9525">
                       <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
+                        <a:schemeClr val="lt1">
+                          <a:lumMod val="95000"/>
+                          <a:alpha val="54000"/>
                         </a:schemeClr>
                       </a:solidFill>
-                      <a:round/>
                     </a:ln>
                     <a:effectLst/>
                   </c:spPr>
@@ -1070,7 +1182,6 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-A088-4DD4-9147-951FA4D70B40}"/>
@@ -1078,7 +1189,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="1"/>
           <c:showCatName val="0"/>
@@ -1086,10 +1196,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:smooth val="0"/>
+        <c:gapWidth val="100"/>
+        <c:overlap val="-24"/>
         <c:axId val="1225796880"/>
         <c:axId val="1225797360"/>
-      </c:lineChart>
+      </c:barChart>
       <c:catAx>
         <c:axId val="1225796880"/>
         <c:scaling>
@@ -1103,11 +1214,11 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -1121,9 +1232,8 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -1166,9 +1276,8 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -1191,37 +1300,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -1234,17 +1312,28 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
     </a:ln>
     <a:effectLst/>
   </c:spPr>
@@ -1269,7 +1358,6 @@
         <c14:dropZoneFilter val="1"/>
         <c14:dropZoneCategories val="1"/>
         <c14:dropZoneData val="1"/>
-        <c14:dropZoneSeries val="1"/>
         <c14:dropZonesVisible val="1"/>
       </c14:pivotOptions>
     </c:ext>
@@ -1307,13 +1395,19 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="95000"/>
                   </a:schemeClr>
                 </a:solidFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                    <a:prstClr val="black">
+                      <a:alpha val="40000"/>
+                    </a:prstClr>
+                  </a:outerShdw>
+                </a:effectLst>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
@@ -1339,13 +1433,19 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
                 </a:schemeClr>
               </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -1359,51 +1459,8 @@
     <c:pivotFmts>
       <c:pivotFmt>
         <c:idx val="0"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln w="19050">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
           <c:dLblPos val="bestFit"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="1"/>
@@ -1419,30 +1476,60 @@
       <c:pivotFmt>
         <c:idx val="1"/>
         <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln w="19050">
-            <a:solidFill>
-              <a:schemeClr val="lt1"/>
-            </a:solidFill>
+          <a:gradFill rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="accent6">
+                  <a:satMod val="103000"/>
+                  <a:lumMod val="102000"/>
+                  <a:tint val="94000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="50000">
+                <a:schemeClr val="accent6">
+                  <a:satMod val="110000"/>
+                  <a:lumMod val="100000"/>
+                  <a:shade val="100000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="99000"/>
+                  <a:satMod val="120000"/>
+                  <a:shade val="78000"/>
+                </a:schemeClr>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="5400000" scaled="0"/>
+          </a:gradFill>
+          <a:ln>
+            <a:noFill/>
           </a:ln>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="none"/>
+          <c:symbol val="circle"/>
+          <c:size val="6"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
           <c:spPr>
-            <a:noFill/>
+            <a:solidFill>
+              <a:sysClr val="window" lastClr="FFFFFF"/>
+            </a:solidFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
               <a:spAutoFit/>
             </a:bodyPr>
             <a:lstStyle/>
@@ -1450,9 +1537,9 @@
               <a:pPr>
                 <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
                     </a:schemeClr>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
@@ -1463,50 +1550,237 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="bestFit"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="1"/>
           <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
+          <c:showPercent val="1"/>
           <c:showBubbleSize val="0"/>
           <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+              <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <a:prstGeom prst="wedgeRectCallout">
+                  <a:avLst/>
+                </a:prstGeom>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+              </c15:spPr>
+            </c:ext>
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="2"/>
         <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln w="19050">
+          <a:gradFill rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="accent6">
+                  <a:satMod val="103000"/>
+                  <a:lumMod val="102000"/>
+                  <a:tint val="94000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="50000">
+                <a:schemeClr val="accent6">
+                  <a:satMod val="110000"/>
+                  <a:lumMod val="100000"/>
+                  <a:shade val="100000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="99000"/>
+                  <a:satMod val="120000"/>
+                  <a:shade val="78000"/>
+                </a:schemeClr>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="5400000" scaled="0"/>
+          </a:gradFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="9.1631375181445679E-2"/>
+              <c:y val="9.4058945016251227E-2"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="lt1"/>
+              <a:sysClr val="window" lastClr="FFFFFF"/>
             </a:solidFill>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+              <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <a:prstGeom prst="wedgeRectCallout">
+                  <a:avLst/>
+                </a:prstGeom>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+              </c15:spPr>
+            </c:ext>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="3"/>
         <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln w="19050">
+          <a:gradFill rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="accent5">
+                  <a:satMod val="103000"/>
+                  <a:lumMod val="102000"/>
+                  <a:tint val="94000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="50000">
+                <a:schemeClr val="accent5">
+                  <a:satMod val="110000"/>
+                  <a:lumMod val="100000"/>
+                  <a:shade val="100000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="99000"/>
+                  <a:satMod val="120000"/>
+                  <a:shade val="78000"/>
+                </a:schemeClr>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="5400000" scaled="0"/>
+          </a:gradFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="-8.4843732296358693E-2"/>
+              <c:y val="2.015548821776815E-2"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="lt1"/>
+              <a:sysClr val="window" lastClr="FFFFFF"/>
             </a:solidFill>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:noAutofit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="dk1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+              <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <a:prstGeom prst="wedgeRectCallout">
+                  <a:avLst/>
+                </a:prstGeom>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+              </c15:spPr>
+              <c15:layout>
+                <c:manualLayout>
+                  <c:w val="0.10890665517956434"/>
+                  <c:h val="0.18283619989165764"/>
+                </c:manualLayout>
+              </c15:layout>
+            </c:ext>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
-      <c:pieChart>
+      <c:doughnutChart>
         <c:varyColors val="1"/>
         <c:ser>
           <c:idx val="0"/>
@@ -1526,15 +1800,42 @@
             <c:idx val="0"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="19050">
-                <a:solidFill>
-                  <a:schemeClr val="lt1"/>
-                </a:solidFill>
+              <a:gradFill rotWithShape="1">
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent6">
+                      <a:satMod val="103000"/>
+                      <a:lumMod val="102000"/>
+                      <a:tint val="94000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="50000">
+                    <a:schemeClr val="accent6">
+                      <a:satMod val="110000"/>
+                      <a:lumMod val="100000"/>
+                      <a:shade val="100000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent6">
+                      <a:lumMod val="99000"/>
+                      <a:satMod val="120000"/>
+                      <a:shade val="78000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="0"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
               </a:ln>
-              <a:effectLst/>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1546,15 +1847,42 @@
             <c:idx val="1"/>
             <c:bubble3D val="0"/>
             <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:ln w="19050">
-                <a:solidFill>
-                  <a:schemeClr val="lt1"/>
-                </a:solidFill>
+              <a:gradFill rotWithShape="1">
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent5">
+                      <a:satMod val="103000"/>
+                      <a:lumMod val="102000"/>
+                      <a:tint val="94000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="50000">
+                    <a:schemeClr val="accent5">
+                      <a:satMod val="110000"/>
+                      <a:lumMod val="100000"/>
+                      <a:shade val="100000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent5">
+                      <a:lumMod val="99000"/>
+                      <a:satMod val="120000"/>
+                      <a:shade val="78000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="0"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
               </a:ln>
-              <a:effectLst/>
+              <a:effectLst>
+                <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="63000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1563,15 +1891,106 @@
             </c:extLst>
           </c:dPt>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="9.1631375181445679E-2"/>
+                  <c:y val="9.4058945016251227E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-9E27-49CE-B742-291B8CE72A30}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-8.4843732296358693E-2"/>
+                  <c:y val="2.015548821776815E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:spPr>
+                <a:solidFill>
+                  <a:sysClr val="window" lastClr="FFFFFF"/>
+                </a:solidFill>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                  <a:noAutofit/>
+                </a:bodyPr>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="dk1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                  <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                    <a:prstGeom prst="wedgeRectCallout">
+                      <a:avLst/>
+                    </a:prstGeom>
+                    <a:noFill/>
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                  </c15:spPr>
+                  <c15:layout>
+                    <c:manualLayout>
+                      <c:w val="0.10890665517956434"/>
+                      <c:h val="0.18283619989165764"/>
+                    </c:manualLayout>
+                  </c15:layout>
+                </c:ext>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-9E27-49CE-B742-291B8CE72A30}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
             <c:spPr>
-              <a:noFill/>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
               <a:ln>
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
               <a:lstStyle/>
@@ -1579,9 +1998,9 @@
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
                       </a:schemeClr>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
@@ -1592,30 +2011,25 @@
                 <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
-            <c:dLblPos val="bestFit"/>
             <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
             <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
+            <c:showPercent val="1"/>
             <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="1"/>
-            <c:leaderLines>
-              <c:spPr>
-                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="35000"/>
-                      <a:lumOff val="65000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:round/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-            </c:leaderLines>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+              </c:ext>
             </c:extLst>
           </c:dLbls>
           <c:cat>
@@ -1654,17 +2068,17 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="bestFit"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
-          <c:showLeaderLines val="1"/>
+          <c:showLeaderLines val="0"/>
         </c:dLbls>
         <c:firstSliceAng val="0"/>
-      </c:pieChart>
+        <c:holeSize val="75"/>
+      </c:doughnutChart>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -1690,9 +2104,8 @@
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -1716,17 +2129,28 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
     </a:ln>
     <a:effectLst/>
   </c:spPr>
@@ -1805,13 +2229,10 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
+  <a:schemeClr val="accent6"/>
+  <a:schemeClr val="accent5"/>
   <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
   <cs:variation/>
   <cs:variation>
     <a:lumMod val="60000"/>
@@ -1845,13 +2266,10 @@
 </file>
 
 <file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
+  <a:schemeClr val="accent6"/>
+  <a:schemeClr val="accent5"/>
   <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
   <cs:variation/>
   <cs:variation>
     <a:lumMod val="60000"/>
@@ -1885,35 +2303,33 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="222">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1921,26 +2337,34 @@
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
     </cs:spPr>
     <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
@@ -1949,9 +2373,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -1970,14 +2393,6 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -1986,20 +2401,20 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
@@ -2008,13 +2423,13 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="28575" cap="rnd">
+      <a:ln w="34925" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -2026,10 +2441,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
@@ -2038,16 +2453,17 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointMarkerLayout size="5"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
@@ -2065,21 +2481,18 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2098,14 +2511,13 @@
           <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -2117,14 +2529,14 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -2138,9 +2550,8 @@
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2154,12 +2565,6 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
@@ -2171,9 +2576,9 @@
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2188,108 +2593,115 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln>
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2301,12 +2713,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -2322,7 +2741,6 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -2331,9 +2749,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2349,14 +2766,13 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -2365,9 +2781,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2379,46 +2794,38 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
   </cs:wall>
 </cs:chartStyle>
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2426,26 +2833,34 @@
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
     </cs:spPr>
     <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
@@ -2454,9 +2869,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2475,14 +2889,6 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -2491,45 +2897,35 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="28575" cap="rnd">
+      <a:ln w="34925" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -2541,33 +2937,31 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -2583,21 +2977,18 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2607,20 +2998,20 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -2631,17 +3022,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -2650,14 +3041,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2669,28 +3059,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2702,111 +3086,118 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln>
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2818,12 +3209,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -2832,14 +3230,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="19050" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -2848,9 +3245,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2860,7 +3256,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -2868,9 +3264,9 @@
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -2881,9 +3277,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2893,48 +3288,40 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="257">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2942,37 +3329,44 @@
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
+    <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -2991,14 +3385,6 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -3007,49 +3393,35 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050">
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="25400">
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="28575" cap="rnd">
+      <a:ln w="34925" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -3061,10 +3433,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
@@ -3073,16 +3445,17 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
@@ -3100,21 +3473,18 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -3133,14 +3503,13 @@
           <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -3152,14 +3521,14 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -3173,9 +3542,8 @@
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3189,12 +3557,6 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
@@ -3206,9 +3568,9 @@
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3223,108 +3585,115 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln>
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3336,12 +3705,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -3357,7 +3733,6 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -3366,9 +3741,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -3384,14 +3758,13 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -3400,9 +3773,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -3414,30 +3786,197 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
   </cs:wall>
 </cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Source">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA7CF1EC-E745-1DCB-E869-C303B0766B0D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Source"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4945380" y="1280161"/>
+              <a:ext cx="1828800" cy="998219"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-IN" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>129540</xdr:colOff>
+      <xdr:colOff>119062</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:rowOff>65314</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>61912</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>160972</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Rectangle 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{919DCDFF-1442-88A6-7994-7AE3CB73B69E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="728662" y="65314"/>
+          <a:ext cx="8640536" cy="6387601"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:gradFill flip="none" rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="75000"/>
+                <a:lumOff val="25000"/>
+                <a:shade val="30000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="75000"/>
+                <a:lumOff val="25000"/>
+                <a:shade val="67500"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="75000"/>
+                <a:lumOff val="25000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="0" scaled="1"/>
+          <a:tileRect/>
+        </a:gradFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-IN" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>396240</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>160020</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>39009</xdr:rowOff>
+      <xdr:colOff>426720</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>46629</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -3452,13 +3991,43 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="739140" y="160020"/>
-          <a:ext cx="1859280" cy="976269"/>
+          <a:off x="1005840" y="1092926"/>
+          <a:ext cx="1859280" cy="989332"/>
           <a:chOff x="739140" y="160020"/>
           <a:chExt cx="1630680" cy="800100"/>
         </a:xfrm>
+        <a:gradFill flip="none" rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="30000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="67500"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="0" scaled="1"/>
+          <a:tileRect/>
+        </a:gradFill>
         <a:effectLst>
-          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" sx="1000" sy="1000" algn="ctr" rotWithShape="0">
             <a:schemeClr val="bg1">
               <a:lumMod val="75000"/>
             </a:schemeClr>
@@ -3484,9 +4053,7 @@
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="bg1"/>
-          </a:solidFill>
+          <a:grpFill/>
           <a:ln>
             <a:gradFill flip="none" rotWithShape="1">
               <a:gsLst>
@@ -3535,12 +4102,9 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="en-IN" sz="1400">
+              <a:rPr lang="en-IN" sz="1400" b="1">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="85000"/>
-                    <a:lumOff val="15000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
               </a:rPr>
               <a:t>Sessions</a:t>
@@ -3567,7 +4131,7 @@
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:noFill/>
+          <a:grpFill/>
         </xdr:spPr>
         <xdr:style>
           <a:lnRef idx="0">
@@ -3593,14 +4157,18 @@
             <a:fld id="{47AFB62C-9460-41C8-BFBE-08748E6C206B}" type="TxLink">
               <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Arial Unicode MS"/>
               </a:rPr>
               <a:pPr algn="ctr"/>
               <a:t>12540</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-IN" sz="3200" b="1"/>
+            <a:endParaRPr lang="en-IN" sz="3200" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -3610,15 +4178,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>236220</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>53340</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>403860</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>38971</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -3633,13 +4201,43 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5280660" y="152400"/>
-          <a:ext cx="1996440" cy="1043940"/>
+          <a:off x="5093426" y="1092926"/>
+          <a:ext cx="1874520" cy="981674"/>
           <a:chOff x="5356860" y="167640"/>
-          <a:chExt cx="1729740" cy="838765"/>
+          <a:chExt cx="1729740" cy="807720"/>
         </a:xfrm>
+        <a:gradFill flip="none" rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="30000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="67500"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="0" scaled="1"/>
+          <a:tileRect/>
+        </a:gradFill>
         <a:effectLst>
-          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" sx="1000" sy="1000" algn="ctr" rotWithShape="0">
             <a:schemeClr val="bg1">
               <a:lumMod val="65000"/>
             </a:schemeClr>
@@ -3665,9 +4263,7 @@
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="bg1"/>
-          </a:solidFill>
+          <a:grpFill/>
           <a:ln>
             <a:gradFill flip="none" rotWithShape="1">
               <a:gsLst>
@@ -3716,12 +4312,9 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="en-IN" sz="1400">
+              <a:rPr lang="en-IN" sz="1400" b="1">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="85000"/>
-                    <a:lumOff val="15000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
               </a:rPr>
               <a:t>Convrsion Rate</a:t>
@@ -3742,13 +4335,13 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="5615940" y="350520"/>
-            <a:ext cx="1280160" cy="655885"/>
+            <a:off x="5676197" y="390041"/>
+            <a:ext cx="1051150" cy="451154"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:noFill/>
+          <a:grpFill/>
         </xdr:spPr>
         <xdr:style>
           <a:lnRef idx="0">
@@ -3766,7 +4359,7 @@
         </xdr:style>
         <xdr:txBody>
           <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
-            <a:spAutoFit/>
+            <a:noAutofit/>
           </a:bodyPr>
           <a:lstStyle/>
           <a:p>
@@ -3774,7 +4367,7 @@
             <a:fld id="{E01E4926-DCB8-4F6C-81F8-262115EFFCF8}" type="TxLink">
               <a:rPr lang="en-US" sz="3600" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
@@ -3783,7 +4376,11 @@
               <a:pPr algn="ctr"/>
               <a:t>4.8%</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-IN" sz="3600" b="1"/>
+            <a:endParaRPr lang="en-IN" sz="3600" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -3792,16 +4389,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>236220</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>350520</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>198120</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -3816,13 +4413,43 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7719060" y="152400"/>
-          <a:ext cx="1943100" cy="1005840"/>
+          <a:off x="7143206" y="1110343"/>
+          <a:ext cx="1752600" cy="978626"/>
           <a:chOff x="7467600" y="175260"/>
           <a:chExt cx="1851660" cy="967740"/>
         </a:xfrm>
+        <a:gradFill flip="none" rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="30000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="67500"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="0" scaled="1"/>
+          <a:tileRect/>
+        </a:gradFill>
         <a:effectLst>
-          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" sx="1000" sy="1000" algn="ctr" rotWithShape="0">
             <a:schemeClr val="bg1">
               <a:lumMod val="65000"/>
             </a:schemeClr>
@@ -3848,9 +4475,7 @@
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="bg1"/>
-          </a:solidFill>
+          <a:grpFill/>
           <a:ln>
             <a:gradFill flip="none" rotWithShape="1">
               <a:gsLst>
@@ -3899,12 +4524,9 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="en-IN" sz="1400">
+              <a:rPr lang="en-IN" sz="1400" b="1">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="85000"/>
-                    <a:lumOff val="15000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
               </a:rPr>
               <a:t>Engagement Rate</a:t>
@@ -3925,15 +4547,13 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="10800000" flipV="1">
-            <a:off x="7916463" y="421986"/>
-            <a:ext cx="1051560" cy="548640"/>
+            <a:off x="7916463" y="453968"/>
+            <a:ext cx="1051560" cy="516657"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="lt1"/>
-          </a:solidFill>
+          <a:grpFill/>
           <a:ln w="9525" cmpd="sng">
             <a:noFill/>
           </a:ln>
@@ -3960,10 +4580,7 @@
             <a:fld id="{38333DA0-2E6F-4080-8C07-C362E06D3BA9}" type="TxLink">
               <a:rPr lang="en-US" sz="3600" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="85000"/>
-                    <a:lumOff val="15000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
                 <a:ea typeface="Calibri"/>
@@ -3974,10 +4591,7 @@
             </a:fld>
             <a:endParaRPr lang="en-IN" sz="3600" b="1">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="85000"/>
-                  <a:lumOff val="15000"/>
-                </a:schemeClr>
+                <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:endParaRPr>
           </a:p>
@@ -3990,13 +4604,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>617220</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>472440</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>45720</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
@@ -4012,13 +4626,43 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3055620" y="160020"/>
-          <a:ext cx="1851660" cy="982980"/>
+          <a:off x="3055620" y="1085306"/>
+          <a:ext cx="1847306" cy="996043"/>
           <a:chOff x="3055620" y="160020"/>
           <a:chExt cx="1851660" cy="982980"/>
         </a:xfrm>
+        <a:gradFill flip="none" rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="30000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="67500"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="tx1">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="115000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="0" scaled="1"/>
+          <a:tileRect/>
+        </a:gradFill>
         <a:effectLst>
-          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+          <a:outerShdw blurRad="50800" dist="50800" dir="5400000" sx="1000" sy="1000" algn="ctr" rotWithShape="0">
             <a:schemeClr val="bg1">
               <a:lumMod val="75000"/>
             </a:schemeClr>
@@ -4044,9 +4688,7 @@
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="bg1"/>
-          </a:solidFill>
+          <a:grpFill/>
           <a:ln>
             <a:gradFill flip="none" rotWithShape="1">
               <a:gsLst>
@@ -4095,12 +4737,9 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="en-IN" sz="1400">
+              <a:rPr lang="en-IN" sz="1400" b="1">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="85000"/>
-                    <a:lumOff val="15000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
               </a:rPr>
               <a:t>Users</a:t>
@@ -4121,15 +4760,13 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="3383280" y="388620"/>
+            <a:off x="3390900" y="426720"/>
             <a:ext cx="1287780" cy="541020"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
           </a:prstGeom>
-          <a:solidFill>
-            <a:schemeClr val="lt1"/>
-          </a:solidFill>
+          <a:grpFill/>
           <a:ln w="9525" cmpd="sng">
             <a:noFill/>
           </a:ln>
@@ -4156,14 +4793,18 @@
             <a:fld id="{3E974562-B1E2-4F5D-A053-A42367A214E1}" type="TxLink">
               <a:rPr lang="en-US" sz="3600" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Arial Unicode MS"/>
               </a:rPr>
               <a:pPr algn="ctr"/>
               <a:t>9870</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-IN" sz="3600" b="1"/>
+            <a:endParaRPr lang="en-IN" sz="3600" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -4172,16 +4813,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>140970</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>396240</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>102870</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>182880</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>500418</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4208,16 +4849,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>137160</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>392429</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>327660</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>522514</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4244,16 +4885,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>224790</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>137160</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>102358</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>102927</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>129540</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>170597</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>156267</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4278,11 +4919,208 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>119062</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>174625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>230187</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="TextBox 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3451F127-EC1B-949E-7A6D-8D57CAED9639}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1952625" y="357188"/>
+          <a:ext cx="5778500" cy="404812"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:grpFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="b" anchorCtr="0">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="en-IN" sz="3200" b="1" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Arial Unicode MS"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>277812</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>103188</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>587375</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="TextBox 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9F6B01E-B152-C887-FDFC-2583457244BD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2111375" y="468313"/>
+          <a:ext cx="5976938" cy="309562"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:grpFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="b" anchorCtr="0">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="en-IN" sz="3200" b="1" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Arial Unicode MS"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>452437</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>15875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="TextBox 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{001F8082-BC96-75AD-0E59-46D784B46535}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2286000" y="381000"/>
+          <a:ext cx="5548313" cy="325438"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="b" anchorCtr="0">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="2000" b="1" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="Arial Unicode MS"/>
+            </a:rPr>
+            <a:t>Website performance analysis </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4324,7 +5162,7 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
+      <x14:pivotCacheDefinition pivotCacheId="925218702"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -4408,7 +5246,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4B0C8D7E-E0B9-498D-A2E7-E27E5E326AFF}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4B0C8D7E-E0B9-498D-A2E7-E27E5E326AFF}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField showAll="0"/>
@@ -4469,7 +5307,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D783F0EE-E993-4B0B-B4AD-089A2E3D8129}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D783F0EE-E993-4B0B-B4AD-089A2E3D8129}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="18">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField axis="axisRow" showAll="0">
@@ -4530,7 +5368,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FE53E59E-A09B-481B-A49E-080D7C76A00C}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FE53E59E-A09B-481B-A49E-080D7C76A00C}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField showAll="0"/>
@@ -4612,6 +5450,28 @@
     </ext>
   </extLst>
 </pivotTableDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Source" xr10:uid="{EFF90958-C38C-4BF9-90B1-4CB4F2EDBAA9}" sourceName="Source">
+  <pivotTables>
+    <pivotTable tabId="4" name="PivotTable3"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="925218702">
+      <items count="2">
+        <i x="0" s="1"/>
+        <i x="1" s="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="Source" xr10:uid="{27454F85-4AA6-4284-9EAA-3DD8A364210E}" cache="Slicer_Source" caption="Source" rowHeight="234950"/>
+</slicers>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4899,7 +5759,40 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:txDef>
+      <a:spPr>
+        <a:grpFill/>
+      </a:spPr>
+      <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="b" anchorCtr="0">
+        <a:noAutofit/>
+      </a:bodyPr>
+      <a:lstStyle>
+        <a:defPPr algn="ctr">
+          <a:defRPr sz="3200" b="1" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Arial Unicode MS"/>
+          </a:defRPr>
+        </a:defPPr>
+      </a:lstStyle>
+      <a:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:txDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
@@ -4930,7 +5823,7 @@
       <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="9">
         <v>6400</v>
       </c>
     </row>
@@ -4938,7 +5831,7 @@
       <c r="A5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="9">
         <v>6140</v>
       </c>
     </row>
@@ -4946,12 +5839,20 @@
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="9">
         <v>12540</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
+      <x14:slicerList>
+        <x14:slicer r:id="rId3"/>
+      </x14:slicerList>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -5022,7 +5923,7 @@
       <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="9">
         <v>5400</v>
       </c>
     </row>
@@ -5030,7 +5931,7 @@
       <c r="A5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="9">
         <v>7140</v>
       </c>
     </row>
@@ -5038,7 +5939,7 @@
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="9">
         <v>12540</v>
       </c>
     </row>
@@ -5320,14 +6221,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{638797E5-C422-4A01-A61C-1B8AA087E31A}">
-  <dimension ref="E5"/>
+  <dimension ref="E10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="5" max="5" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="5:5" ht="14.4" customHeight="1">
-      <c r="E5" s="6"/>
+    <row r="10" spans="5:5" ht="14.4" customHeight="1">
+      <c r="E10" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>